<commit_message>
Add Uzbekistan official shadow economy (% GDP) from Uzbek Statistics Committee
- Source: Uzbekistan National Statistics Committee 'hidden economy' dataset
  (code 1.01.08.0014), billion soum, converted to % of GDP via nominal GDP (WB)
- Uzbekistan shadow economy ~7-8% of GDP, 2011-2020 (official NOE methodology)
- Added as SEPARATE column SHADOW_OFFICIAL (not mixed with DGE: ~7-8% official NOE
  is not comparable to ~33-43% DGE/MIMIC academic estimates)
</commit_message>
<xml_diff>
--- a/DFS_data_IMPUTED.xlsx
+++ b/DFS_data_IMPUTED.xlsx
@@ -40,7 +40,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +72,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -99,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +115,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -558,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U51"/>
+  <dimension ref="A1:V51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -582,6 +588,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -690,6 +697,11 @@
           <t>INST</t>
         </is>
       </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>SHADOW_OFFICIAL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -715,7 +727,7 @@
       <c r="G2" s="5" t="n">
         <v>42.1051</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="5" t="n">
         <v>33.5229</v>
       </c>
       <c r="I2" s="5" t="n">
@@ -757,6 +769,7 @@
       <c r="U2" s="5" t="n">
         <v>-0.4487</v>
       </c>
+      <c r="V2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -782,7 +795,7 @@
       <c r="G3" s="5" t="n">
         <v>46.0392</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="5" t="n">
         <v>39.5934</v>
       </c>
       <c r="I3" s="5" t="n">
@@ -824,6 +837,7 @@
       <c r="U3" s="5" t="n">
         <v>-0.4892</v>
       </c>
+      <c r="V3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -849,7 +863,7 @@
       <c r="G4" s="5" t="n">
         <v>49.9733</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="5" t="n">
         <v>43.087</v>
       </c>
       <c r="I4" s="5" t="n">
@@ -891,6 +905,7 @@
       <c r="U4" s="5" t="n">
         <v>-0.5085</v>
       </c>
+      <c r="V4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -958,6 +973,7 @@
       <c r="U5" s="5" t="n">
         <v>-0.373</v>
       </c>
+      <c r="V5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1025,6 +1041,7 @@
       <c r="U6" s="5" t="n">
         <v>-0.2817</v>
       </c>
+      <c r="V6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1092,6 +1109,7 @@
       <c r="U7" s="5" t="n">
         <v>-0.3231</v>
       </c>
+      <c r="V7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1159,6 +1177,7 @@
       <c r="U8" s="5" t="n">
         <v>-0.1891</v>
       </c>
+      <c r="V8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1226,6 +1245,7 @@
       <c r="U9" s="5" t="n">
         <v>-0.1576</v>
       </c>
+      <c r="V9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1293,6 +1313,7 @@
       <c r="U10" s="5" t="n">
         <v>-0.1592</v>
       </c>
+      <c r="V10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1360,6 +1381,7 @@
       <c r="U11" s="5" t="n">
         <v>-0.1807</v>
       </c>
+      <c r="V11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1379,13 +1401,13 @@
       <c r="E12" s="5" t="n">
         <v>37.1967</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="5" t="n">
         <v>17.8388</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>3.7573</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="5" t="n">
@@ -1427,6 +1449,7 @@
       <c r="U12" s="5" t="n">
         <v>-0.7053</v>
       </c>
+      <c r="V12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1446,13 +1469,13 @@
       <c r="E13" s="5" t="n">
         <v>36.9522</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="5" t="n">
         <v>18.7272</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>8.6617</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="5" t="n">
         <v>2.3741</v>
       </c>
       <c r="I13" s="5" t="n">
@@ -1494,6 +1517,7 @@
       <c r="U13" s="5" t="n">
         <v>-0.7169</v>
       </c>
+      <c r="V13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1513,13 +1537,13 @@
       <c r="E14" s="5" t="n">
         <v>42.1473</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="5" t="n">
         <v>18.1138</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>13.5662</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="5" t="n">
         <v>9.4552</v>
       </c>
       <c r="I14" s="5" t="n">
@@ -1561,6 +1585,7 @@
       <c r="U14" s="5" t="n">
         <v>-0.6919</v>
       </c>
+      <c r="V14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1628,6 +1653,7 @@
       <c r="U15" s="5" t="n">
         <v>-0.6804</v>
       </c>
+      <c r="V15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1695,6 +1721,7 @@
       <c r="U16" s="5" t="n">
         <v>-0.6988</v>
       </c>
+      <c r="V16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1762,6 +1789,7 @@
       <c r="U17" s="5" t="n">
         <v>-0.5957</v>
       </c>
+      <c r="V17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1829,6 +1857,7 @@
       <c r="U18" s="5" t="n">
         <v>-0.5036</v>
       </c>
+      <c r="V18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1896,6 +1925,7 @@
       <c r="U19" s="5" t="n">
         <v>-0.5212</v>
       </c>
+      <c r="V19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1963,6 +1993,7 @@
       <c r="U20" s="5" t="n">
         <v>-0.5798</v>
       </c>
+      <c r="V20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2030,6 +2061,7 @@
       <c r="U21" s="5" t="n">
         <v>-0.607</v>
       </c>
+      <c r="V21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2055,7 +2087,7 @@
       <c r="G22" s="5" t="n">
         <v>2.5349</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I22" s="5" t="n">
@@ -2097,6 +2129,7 @@
       <c r="U22" s="5" t="n">
         <v>-1.1105</v>
       </c>
+      <c r="V22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2122,7 +2155,7 @@
       <c r="G23" s="5" t="n">
         <v>5.5097</v>
       </c>
-      <c r="H23" s="6" t="n">
+      <c r="H23" s="5" t="n">
         <v>2.3735</v>
       </c>
       <c r="I23" s="5" t="n">
@@ -2164,6 +2197,7 @@
       <c r="U23" s="5" t="n">
         <v>-1.0899</v>
       </c>
+      <c r="V23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2189,7 +2223,7 @@
       <c r="G24" s="5" t="n">
         <v>8.484400000000001</v>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H24" s="5" t="n">
         <v>6.082</v>
       </c>
       <c r="I24" s="5" t="n">
@@ -2231,6 +2265,7 @@
       <c r="U24" s="5" t="n">
         <v>-1.1126</v>
       </c>
+      <c r="V24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2298,6 +2333,7 @@
       <c r="U25" s="5" t="n">
         <v>-1.041</v>
       </c>
+      <c r="V25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2365,6 +2401,7 @@
       <c r="U26" s="5" t="n">
         <v>-1.0065</v>
       </c>
+      <c r="V26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2432,6 +2469,7 @@
       <c r="U27" s="5" t="n">
         <v>-1.0278</v>
       </c>
+      <c r="V27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2475,7 +2513,7 @@
       <c r="M28" s="5" t="n">
         <v>7.035</v>
       </c>
-      <c r="N28" s="6" t="n">
+      <c r="N28" s="5" t="n">
         <v>2.7817</v>
       </c>
       <c r="O28" s="5" t="n">
@@ -2497,8 +2535,9 @@
         <v>-1.1642</v>
       </c>
       <c r="U28" s="5" t="n">
-        <v>-0.9774</v>
-      </c>
+        <v>-0.9775</v>
+      </c>
+      <c r="V28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2542,7 +2581,7 @@
       <c r="M29" s="5" t="n">
         <v>7.028</v>
       </c>
-      <c r="N29" s="6" t="n">
+      <c r="N29" s="5" t="n">
         <v>3.5254</v>
       </c>
       <c r="O29" s="5" t="n">
@@ -2566,6 +2605,7 @@
       <c r="U29" s="5" t="n">
         <v>-0.9348</v>
       </c>
+      <c r="V29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2609,7 +2649,7 @@
       <c r="M30" s="5" t="n">
         <v>7.026</v>
       </c>
-      <c r="N30" s="6" t="n">
+      <c r="N30" s="5" t="n">
         <v>3.408</v>
       </c>
       <c r="O30" s="5" t="n">
@@ -2633,6 +2673,7 @@
       <c r="U30" s="5" t="n">
         <v>-1.0236</v>
       </c>
+      <c r="V30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2676,7 +2717,7 @@
       <c r="M31" s="5" t="n">
         <v>7.576</v>
       </c>
-      <c r="N31" s="6" t="n">
+      <c r="N31" s="5" t="n">
         <v>8.7949</v>
       </c>
       <c r="O31" s="5" t="n">
@@ -2700,6 +2741,7 @@
       <c r="U31" s="5" t="n">
         <v>-1.0238</v>
       </c>
+      <c r="V31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2715,16 +2757,16 @@
       <c r="E32" s="5" t="n">
         <v>36.7918</v>
       </c>
-      <c r="F32" s="6" t="n">
+      <c r="F32" s="5" t="n">
         <v>14.9552</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>0.4049</v>
       </c>
-      <c r="H32" s="6" t="n">
+      <c r="H32" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I32" s="6" t="n">
+      <c r="I32" s="5" t="n">
         <v>25.6222</v>
       </c>
       <c r="J32" s="5" t="n">
@@ -2739,10 +2781,10 @@
       <c r="M32" s="5" t="n">
         <v>4.003</v>
       </c>
-      <c r="N32" s="6" t="n">
+      <c r="N32" s="5" t="n">
         <v>13.8329</v>
       </c>
-      <c r="O32" s="6" t="n">
+      <c r="O32" s="5" t="n">
         <v>22.4372</v>
       </c>
       <c r="P32" s="5" t="n">
@@ -2763,6 +2805,7 @@
       <c r="U32" s="5" t="n">
         <v>-1.626</v>
       </c>
+      <c r="V32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2778,16 +2821,16 @@
       <c r="E33" s="5" t="n">
         <v>36.2132</v>
       </c>
-      <c r="F33" s="6" t="n">
+      <c r="F33" s="5" t="n">
         <v>15.4676</v>
       </c>
       <c r="G33" s="5" t="n">
         <v>7.1002</v>
       </c>
-      <c r="H33" s="6" t="n">
+      <c r="H33" s="5" t="n">
         <v>0.0112</v>
       </c>
-      <c r="I33" s="6" t="n">
+      <c r="I33" s="5" t="n">
         <v>27.0539</v>
       </c>
       <c r="J33" s="5" t="n">
@@ -2802,10 +2845,10 @@
       <c r="M33" s="5" t="n">
         <v>3.994</v>
       </c>
-      <c r="N33" s="6" t="n">
+      <c r="N33" s="5" t="n">
         <v>12.6123</v>
       </c>
-      <c r="O33" s="6" t="n">
+      <c r="O33" s="5" t="n">
         <v>20.2774</v>
       </c>
       <c r="P33" s="5" t="n">
@@ -2826,6 +2869,7 @@
       <c r="U33" s="5" t="n">
         <v>-1.6012</v>
       </c>
+      <c r="V33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2841,16 +2885,16 @@
       <c r="E34" s="5" t="n">
         <v>35.6764</v>
       </c>
-      <c r="F34" s="6" t="n">
+      <c r="F34" s="5" t="n">
         <v>14.7515</v>
       </c>
       <c r="G34" s="5" t="n">
         <v>13.7954</v>
       </c>
-      <c r="H34" s="6" t="n">
+      <c r="H34" s="5" t="n">
         <v>7.2959</v>
       </c>
-      <c r="I34" s="6" t="n">
+      <c r="I34" s="5" t="n">
         <v>27.723</v>
       </c>
       <c r="J34" s="5" t="n">
@@ -2865,10 +2909,10 @@
       <c r="M34" s="5" t="n">
         <v>3.993</v>
       </c>
-      <c r="N34" s="6" t="n">
+      <c r="N34" s="5" t="n">
         <v>11.6217</v>
       </c>
-      <c r="O34" s="6" t="n">
+      <c r="O34" s="5" t="n">
         <v>17.9722</v>
       </c>
       <c r="P34" s="5" t="n">
@@ -2889,6 +2933,7 @@
       <c r="U34" s="5" t="n">
         <v>-1.6093</v>
       </c>
+      <c r="V34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2904,16 +2949,16 @@
       <c r="E35" s="5" t="n">
         <v>35.1884</v>
       </c>
-      <c r="F35" s="6" t="n">
+      <c r="F35" s="5" t="n">
         <v>14.9678</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>20.4907</v>
-      </c>
-      <c r="H35" s="6" t="n">
+        <v>20.4906</v>
+      </c>
+      <c r="H35" s="5" t="n">
         <v>14.1563</v>
       </c>
-      <c r="I35" s="6" t="n">
+      <c r="I35" s="5" t="n">
         <v>31.325</v>
       </c>
       <c r="J35" s="5" t="n">
@@ -2928,10 +2973,10 @@
       <c r="M35" s="5" t="n">
         <v>4.005</v>
       </c>
-      <c r="N35" s="6" t="n">
+      <c r="N35" s="5" t="n">
         <v>9.6305</v>
       </c>
-      <c r="O35" s="6" t="n">
+      <c r="O35" s="5" t="n">
         <v>15.4037</v>
       </c>
       <c r="P35" s="5" t="n">
@@ -2952,6 +2997,7 @@
       <c r="U35" s="5" t="n">
         <v>-1.5953</v>
       </c>
+      <c r="V35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2967,16 +3013,16 @@
       <c r="E36" s="5" t="n">
         <v>34.7667</v>
       </c>
-      <c r="F36" s="6" t="n">
+      <c r="F36" s="5" t="n">
         <v>13.3775</v>
       </c>
       <c r="G36" s="5" t="n">
         <v>27.1859</v>
       </c>
-      <c r="H36" s="6" t="n">
+      <c r="H36" s="5" t="n">
         <v>21.032</v>
       </c>
-      <c r="I36" s="6" t="n">
+      <c r="I36" s="5" t="n">
         <v>31.6656</v>
       </c>
       <c r="J36" s="5" t="n">
@@ -2991,10 +3037,10 @@
       <c r="M36" s="5" t="n">
         <v>4.016</v>
       </c>
-      <c r="N36" s="6" t="n">
+      <c r="N36" s="5" t="n">
         <v>8.1381</v>
       </c>
-      <c r="O36" s="6" t="n">
+      <c r="O36" s="5" t="n">
         <v>12.0247</v>
       </c>
       <c r="P36" s="5" t="n">
@@ -3015,6 +3061,7 @@
       <c r="U36" s="5" t="n">
         <v>-1.5898</v>
       </c>
+      <c r="V36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -3030,16 +3077,16 @@
       <c r="E37" s="5" t="n">
         <v>34.4187</v>
       </c>
-      <c r="F37" s="6" t="n">
+      <c r="F37" s="5" t="n">
         <v>12.8017</v>
       </c>
       <c r="G37" s="5" t="n">
         <v>33.8811</v>
       </c>
-      <c r="H37" s="6" t="n">
+      <c r="H37" s="5" t="n">
         <v>27.7396</v>
       </c>
-      <c r="I37" s="6" t="n">
+      <c r="I37" s="5" t="n">
         <v>34.2678</v>
       </c>
       <c r="J37" s="5" t="n">
@@ -3054,10 +3101,10 @@
       <c r="M37" s="5" t="n">
         <v>4.026</v>
       </c>
-      <c r="N37" s="6" t="n">
+      <c r="N37" s="5" t="n">
         <v>6.8106</v>
       </c>
-      <c r="O37" s="6" t="n">
+      <c r="O37" s="5" t="n">
         <v>9.5593</v>
       </c>
       <c r="P37" s="5" t="n">
@@ -3078,6 +3125,7 @@
       <c r="U37" s="5" t="n">
         <v>-1.6315</v>
       </c>
+      <c r="V37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -3093,7 +3141,7 @@
       <c r="E38" s="5" t="n">
         <v>34.1184</v>
       </c>
-      <c r="F38" s="6" t="n">
+      <c r="F38" s="5" t="n">
         <v>10.7662</v>
       </c>
       <c r="G38" s="5" t="n">
@@ -3102,7 +3150,7 @@
       <c r="H38" s="5" t="n">
         <v>34.2975</v>
       </c>
-      <c r="I38" s="6" t="n">
+      <c r="I38" s="5" t="n">
         <v>33.6906</v>
       </c>
       <c r="J38" s="5" t="n">
@@ -3117,10 +3165,10 @@
       <c r="M38" s="5" t="n">
         <v>4.035</v>
       </c>
-      <c r="N38" s="6" t="n">
+      <c r="N38" s="5" t="n">
         <v>8.4214</v>
       </c>
-      <c r="O38" s="6" t="n">
+      <c r="O38" s="5" t="n">
         <v>8.277200000000001</v>
       </c>
       <c r="P38" s="5" t="n">
@@ -3141,6 +3189,7 @@
       <c r="U38" s="5" t="n">
         <v>-1.6343</v>
       </c>
+      <c r="V38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -3156,16 +3205,16 @@
       <c r="E39" s="5" t="n">
         <v>33.8603</v>
       </c>
-      <c r="F39" s="6" t="n">
+      <c r="F39" s="5" t="n">
         <v>8.904999999999999</v>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="G39" s="5" t="n">
         <v>39.5999</v>
       </c>
-      <c r="H39" s="6" t="n">
+      <c r="H39" s="5" t="n">
         <v>34.2711</v>
       </c>
-      <c r="I39" s="6" t="n">
+      <c r="I39" s="5" t="n">
         <v>33.122</v>
       </c>
       <c r="J39" s="5" t="n">
@@ -3180,10 +3229,10 @@
       <c r="M39" s="5" t="n">
         <v>4.036</v>
       </c>
-      <c r="N39" s="6" t="n">
+      <c r="N39" s="5" t="n">
         <v>10.7646</v>
       </c>
-      <c r="O39" s="6" t="n">
+      <c r="O39" s="5" t="n">
         <v>8.8247</v>
       </c>
       <c r="P39" s="5" t="n">
@@ -3204,6 +3253,7 @@
       <c r="U39" s="5" t="n">
         <v>-1.621</v>
       </c>
+      <c r="V39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -3219,16 +3269,16 @@
       <c r="E40" s="5" t="n">
         <v>33.6193</v>
       </c>
-      <c r="F40" s="6" t="n">
+      <c r="F40" s="5" t="n">
         <v>8.4983</v>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="G40" s="5" t="n">
         <v>41.4012</v>
       </c>
-      <c r="H40" s="6" t="n">
+      <c r="H40" s="5" t="n">
         <v>35.7655</v>
       </c>
-      <c r="I40" s="6" t="n">
+      <c r="I40" s="5" t="n">
         <v>37.544</v>
       </c>
       <c r="J40" s="5" t="n">
@@ -3243,10 +3293,10 @@
       <c r="M40" s="5" t="n">
         <v>4.035</v>
       </c>
-      <c r="N40" s="6" t="n">
+      <c r="N40" s="5" t="n">
         <v>11.0642</v>
       </c>
-      <c r="O40" s="6" t="n">
+      <c r="O40" s="5" t="n">
         <v>8.382300000000001</v>
       </c>
       <c r="P40" s="5" t="n">
@@ -3267,6 +3317,7 @@
       <c r="U40" s="5" t="n">
         <v>-1.6521</v>
       </c>
+      <c r="V40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -3282,16 +3333,16 @@
       <c r="E41" s="5" t="n">
         <v>33.0787</v>
       </c>
-      <c r="F41" s="6" t="n">
+      <c r="F41" s="5" t="n">
         <v>7.8406</v>
       </c>
-      <c r="G41" s="6" t="n">
+      <c r="G41" s="5" t="n">
         <v>43.6948</v>
       </c>
-      <c r="H41" s="6" t="n">
+      <c r="H41" s="5" t="n">
         <v>37.6165</v>
       </c>
-      <c r="I41" s="6" t="n">
+      <c r="I41" s="5" t="n">
         <v>42.2997</v>
       </c>
       <c r="J41" s="5" t="n">
@@ -3306,10 +3357,10 @@
       <c r="M41" s="5" t="n">
         <v>4.489</v>
       </c>
-      <c r="N41" s="6" t="n">
+      <c r="N41" s="5" t="n">
         <v>11.3652</v>
       </c>
-      <c r="O41" s="6" t="n">
+      <c r="O41" s="5" t="n">
         <v>7.8708</v>
       </c>
       <c r="P41" s="5" t="n">
@@ -3330,6 +3381,7 @@
       <c r="U41" s="5" t="n">
         <v>-1.6206</v>
       </c>
+      <c r="V41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -3351,10 +3403,10 @@
       <c r="G42" s="5" t="n">
         <v>22.5039</v>
       </c>
-      <c r="H42" s="6" t="n">
+      <c r="H42" s="5" t="n">
         <v>17.1347</v>
       </c>
-      <c r="I42" s="6" t="n">
+      <c r="I42" s="5" t="n">
         <v>8.470000000000001</v>
       </c>
       <c r="J42" s="5" t="n">
@@ -3392,6 +3444,9 @@
       </c>
       <c r="U42" s="5" t="n">
         <v>-1.472</v>
+      </c>
+      <c r="V42" s="8" t="n">
+        <v>7.57</v>
       </c>
     </row>
     <row r="43">
@@ -3414,10 +3469,10 @@
       <c r="G43" s="5" t="n">
         <v>28.5726</v>
       </c>
-      <c r="H43" s="6" t="n">
+      <c r="H43" s="5" t="n">
         <v>24.1966</v>
       </c>
-      <c r="I43" s="6" t="n">
+      <c r="I43" s="5" t="n">
         <v>7.0451</v>
       </c>
       <c r="J43" s="5" t="n">
@@ -3455,6 +3510,9 @@
       </c>
       <c r="U43" s="5" t="n">
         <v>-1.3248</v>
+      </c>
+      <c r="V43" s="8" t="n">
+        <v>7.33</v>
       </c>
     </row>
     <row r="44">
@@ -3477,10 +3535,10 @@
       <c r="G44" s="5" t="n">
         <v>34.6413</v>
       </c>
-      <c r="H44" s="6" t="n">
+      <c r="H44" s="5" t="n">
         <v>30.9365</v>
       </c>
-      <c r="I44" s="6" t="n">
+      <c r="I44" s="5" t="n">
         <v>8.919600000000001</v>
       </c>
       <c r="J44" s="5" t="n">
@@ -3518,6 +3576,9 @@
       </c>
       <c r="U44" s="5" t="n">
         <v>-1.2945</v>
+      </c>
+      <c r="V44" s="8" t="n">
+        <v>8.02</v>
       </c>
     </row>
     <row r="45">
@@ -3582,6 +3643,9 @@
       <c r="U45" s="5" t="n">
         <v>-1.2757</v>
       </c>
+      <c r="V45" s="8" t="n">
+        <v>8.119999999999999</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3645,6 +3709,9 @@
       <c r="U46" s="5" t="n">
         <v>-1.2503</v>
       </c>
+      <c r="V46" s="8" t="n">
+        <v>7.63</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3708,6 +3775,9 @@
       <c r="U47" s="5" t="n">
         <v>-1.2217</v>
       </c>
+      <c r="V47" s="8" t="n">
+        <v>7.66</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3771,6 +3841,9 @@
       <c r="U48" s="5" t="n">
         <v>-1.1445</v>
       </c>
+      <c r="V48" s="8" t="n">
+        <v>6.99</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3834,6 +3907,9 @@
       <c r="U49" s="5" t="n">
         <v>-1.0216</v>
       </c>
+      <c r="V49" s="8" t="n">
+        <v>6.88</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3897,6 +3973,9 @@
       <c r="U50" s="5" t="n">
         <v>-0.9327</v>
       </c>
+      <c r="V50" s="8" t="n">
+        <v>7.43</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3958,7 +4037,10 @@
         <v>-0.9126</v>
       </c>
       <c r="U51" s="5" t="n">
-        <v>-0.9675</v>
+        <v>-0.9676</v>
+      </c>
+      <c r="V51" s="8" t="n">
+        <v>6.49</v>
       </c>
     </row>
   </sheetData>
@@ -3972,7 +4054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U201"/>
+  <dimension ref="A1:V201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3996,6 +4078,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4104,6 +4187,11 @@
           <t>INST</t>
         </is>
       </c>
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>SHADOW_OFFICIAL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -4129,7 +4217,7 @@
       <c r="G2" s="5" t="n">
         <v>28.2681</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="H2" s="5" t="n">
         <v>6.2748</v>
       </c>
       <c r="I2" s="5" t="n">
@@ -4171,6 +4259,7 @@
       <c r="U2" s="5" t="n">
         <v>-0.1227</v>
       </c>
+      <c r="V2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -4196,7 +4285,7 @@
       <c r="G3" s="5" t="n">
         <v>31.5075</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="H3" s="5" t="n">
         <v>12.2365</v>
       </c>
       <c r="I3" s="5" t="n">
@@ -4238,6 +4327,7 @@
       <c r="U3" s="5" t="n">
         <v>-0.2429</v>
       </c>
+      <c r="V3" s="7" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -4263,7 +4353,7 @@
       <c r="G4" s="5" t="n">
         <v>34.747</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="H4" s="5" t="n">
         <v>16.6902</v>
       </c>
       <c r="I4" s="5" t="n">
@@ -4305,6 +4395,7 @@
       <c r="U4" s="5" t="n">
         <v>-0.2726</v>
       </c>
+      <c r="V4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -4372,6 +4463,7 @@
       <c r="U5" s="5" t="n">
         <v>-0.1099</v>
       </c>
+      <c r="V5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -4439,6 +4531,7 @@
       <c r="U6" s="5" t="n">
         <v>-0.0912</v>
       </c>
+      <c r="V6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -4506,6 +4599,7 @@
       <c r="U7" s="5" t="n">
         <v>-0.0709</v>
       </c>
+      <c r="V7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -4573,6 +4667,7 @@
       <c r="U8" s="5" t="n">
         <v>-0.0476</v>
       </c>
+      <c r="V8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -4640,6 +4735,7 @@
       <c r="U9" s="5" t="n">
         <v>-0.0302</v>
       </c>
+      <c r="V9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -4666,7 +4762,7 @@
         <v>42.0947</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>31.6876</v>
+        <v>31.6877</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>30.1141</v>
@@ -4707,6 +4803,7 @@
       <c r="U10" s="5" t="n">
         <v>-0.0998</v>
       </c>
+      <c r="V10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -4774,6 +4871,7 @@
       <c r="U11" s="5" t="n">
         <v>-0.1381</v>
       </c>
+      <c r="V11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -4799,7 +4897,7 @@
       <c r="G12" s="5" t="n">
         <v>17.4869</v>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H12" s="5" t="n">
         <v>2.4954</v>
       </c>
       <c r="I12" s="5" t="n">
@@ -4841,6 +4939,7 @@
       <c r="U12" s="5" t="n">
         <v>-0.008</v>
       </c>
+      <c r="V12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -4866,7 +4965,7 @@
       <c r="G13" s="5" t="n">
         <v>17.5476</v>
       </c>
-      <c r="H13" s="6" t="n">
+      <c r="H13" s="5" t="n">
         <v>5.8449</v>
       </c>
       <c r="I13" s="5" t="n">
@@ -4908,6 +5007,7 @@
       <c r="U13" s="5" t="n">
         <v>0.0254</v>
       </c>
+      <c r="V13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -4933,7 +5033,7 @@
       <c r="G14" s="5" t="n">
         <v>17.6084</v>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H14" s="5" t="n">
         <v>9.801500000000001</v>
       </c>
       <c r="I14" s="5" t="n">
@@ -4975,6 +5075,7 @@
       <c r="U14" s="5" t="n">
         <v>0.0211</v>
       </c>
+      <c r="V14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -5042,6 +5143,7 @@
       <c r="U15" s="5" t="n">
         <v>-0.1455</v>
       </c>
+      <c r="V15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -5109,6 +5211,7 @@
       <c r="U16" s="5" t="n">
         <v>-0.0917</v>
       </c>
+      <c r="V16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -5176,6 +5279,7 @@
       <c r="U17" s="5" t="n">
         <v>-0.0328</v>
       </c>
+      <c r="V17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -5243,6 +5347,7 @@
       <c r="U18" s="5" t="n">
         <v>-0.0267</v>
       </c>
+      <c r="V18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -5310,6 +5415,7 @@
       <c r="U19" s="5" t="n">
         <v>0.0333</v>
       </c>
+      <c r="V19" s="7" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -5377,6 +5483,7 @@
       <c r="U20" s="5" t="n">
         <v>0.0052</v>
       </c>
+      <c r="V20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -5442,8 +5549,9 @@
         <v>-0.0752</v>
       </c>
       <c r="U21" s="5" t="n">
-        <v>0.0665</v>
-      </c>
+        <v>0.0664</v>
+      </c>
+      <c r="V21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -5469,7 +5577,7 @@
       <c r="G22" s="5" t="n">
         <v>14.9009</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H22" s="5" t="n">
         <v>1.2645</v>
       </c>
       <c r="I22" s="5" t="n">
@@ -5511,6 +5619,7 @@
       <c r="U22" s="5" t="n">
         <v>-0.6012999999999999</v>
       </c>
+      <c r="V22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -5536,7 +5645,7 @@
       <c r="G23" s="5" t="n">
         <v>19.6511</v>
       </c>
-      <c r="H23" s="6" t="n">
+      <c r="H23" s="5" t="n">
         <v>8.865</v>
       </c>
       <c r="I23" s="5" t="n">
@@ -5578,6 +5687,7 @@
       <c r="U23" s="5" t="n">
         <v>-0.6205000000000001</v>
       </c>
+      <c r="V23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -5603,7 +5713,7 @@
       <c r="G24" s="5" t="n">
         <v>24.4013</v>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H24" s="5" t="n">
         <v>15.3103</v>
       </c>
       <c r="I24" s="5" t="n">
@@ -5645,6 +5755,7 @@
       <c r="U24" s="5" t="n">
         <v>-0.5276999999999999</v>
       </c>
+      <c r="V24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -5712,6 +5823,7 @@
       <c r="U25" s="5" t="n">
         <v>-0.4625</v>
       </c>
+      <c r="V25" s="7" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -5779,6 +5891,7 @@
       <c r="U26" s="5" t="n">
         <v>-0.4836</v>
       </c>
+      <c r="V26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -5846,6 +5959,7 @@
       <c r="U27" s="5" t="n">
         <v>-0.445</v>
       </c>
+      <c r="V27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -5913,6 +6027,7 @@
       <c r="U28" s="5" t="n">
         <v>-0.4491</v>
       </c>
+      <c r="V28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -5980,6 +6095,7 @@
       <c r="U29" s="5" t="n">
         <v>-0.4269</v>
       </c>
+      <c r="V29" s="7" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -6047,6 +6163,7 @@
       <c r="U30" s="5" t="n">
         <v>-0.3886</v>
       </c>
+      <c r="V30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -6114,6 +6231,7 @@
       <c r="U31" s="5" t="n">
         <v>-0.3619</v>
       </c>
+      <c r="V31" s="7" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -6139,7 +6257,7 @@
       <c r="G32" s="5" t="n">
         <v>58.602</v>
       </c>
-      <c r="H32" s="6" t="n">
+      <c r="H32" s="5" t="n">
         <v>48.0114</v>
       </c>
       <c r="I32" s="5" t="n">
@@ -6181,6 +6299,7 @@
       <c r="U32" s="5" t="n">
         <v>-1.1651</v>
       </c>
+      <c r="V32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -6206,7 +6325,7 @@
       <c r="G33" s="5" t="n">
         <v>63.063</v>
       </c>
-      <c r="H33" s="6" t="n">
+      <c r="H33" s="5" t="n">
         <v>53.637</v>
       </c>
       <c r="I33" s="5" t="n">
@@ -6248,6 +6367,7 @@
       <c r="U33" s="5" t="n">
         <v>-0.884</v>
       </c>
+      <c r="V33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -6273,7 +6393,7 @@
       <c r="G34" s="5" t="n">
         <v>67.524</v>
       </c>
-      <c r="H34" s="6" t="n">
+      <c r="H34" s="5" t="n">
         <v>60.7453</v>
       </c>
       <c r="I34" s="5" t="n">
@@ -6315,6 +6435,7 @@
       <c r="U34" s="5" t="n">
         <v>-0.929</v>
       </c>
+      <c r="V34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -6382,6 +6503,7 @@
       <c r="U35" s="5" t="n">
         <v>-0.821</v>
       </c>
+      <c r="V35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -6449,6 +6571,7 @@
       <c r="U36" s="5" t="n">
         <v>-0.8671</v>
       </c>
+      <c r="V36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -6516,6 +6639,7 @@
       <c r="U37" s="5" t="n">
         <v>-0.8134</v>
       </c>
+      <c r="V37" s="7" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -6583,6 +6707,7 @@
       <c r="U38" s="5" t="n">
         <v>-0.8208</v>
       </c>
+      <c r="V38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -6605,10 +6730,10 @@
       <c r="F39" s="5" t="n">
         <v>14.6726</v>
       </c>
-      <c r="G39" s="6" t="n">
+      <c r="G39" s="5" t="n">
         <v>75.11</v>
       </c>
-      <c r="H39" s="6" t="n">
+      <c r="H39" s="5" t="n">
         <v>74.55070000000001</v>
       </c>
       <c r="I39" s="5" t="n">
@@ -6650,6 +6775,7 @@
       <c r="U39" s="5" t="n">
         <v>-0.7607</v>
       </c>
+      <c r="V39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -6672,10 +6798,10 @@
       <c r="F40" s="5" t="n">
         <v>13.3015</v>
       </c>
-      <c r="G40" s="6" t="n">
+      <c r="G40" s="5" t="n">
         <v>78.5087</v>
       </c>
-      <c r="H40" s="6" t="n">
+      <c r="H40" s="5" t="n">
         <v>77.16119999999999</v>
       </c>
       <c r="I40" s="5" t="n">
@@ -6717,6 +6843,7 @@
       <c r="U40" s="5" t="n">
         <v>-0.6509</v>
       </c>
+      <c r="V40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -6739,10 +6866,10 @@
       <c r="F41" s="5" t="n">
         <v>12.0229</v>
       </c>
-      <c r="G41" s="6" t="n">
+      <c r="G41" s="5" t="n">
         <v>82.3403</v>
       </c>
-      <c r="H41" s="6" t="n">
+      <c r="H41" s="5" t="n">
         <v>80.3856</v>
       </c>
       <c r="I41" s="5" t="n">
@@ -6784,6 +6911,7 @@
       <c r="U41" s="5" t="n">
         <v>-0.7716</v>
       </c>
+      <c r="V41" s="7" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -6809,7 +6937,7 @@
       <c r="G42" s="5" t="n">
         <v>56.2116</v>
       </c>
-      <c r="H42" s="6" t="n">
+      <c r="H42" s="5" t="n">
         <v>31.937</v>
       </c>
       <c r="I42" s="5" t="n">
@@ -6849,8 +6977,9 @@
         <v>-0.4173</v>
       </c>
       <c r="U42" s="5" t="n">
-        <v>-0.3445</v>
-      </c>
+        <v>-0.3444</v>
+      </c>
+      <c r="V42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -6876,7 +7005,7 @@
       <c r="G43" s="5" t="n">
         <v>55.0361</v>
       </c>
-      <c r="H43" s="6" t="n">
+      <c r="H43" s="5" t="n">
         <v>32.6299</v>
       </c>
       <c r="I43" s="5" t="n">
@@ -6918,6 +7047,7 @@
       <c r="U43" s="5" t="n">
         <v>-0.1685</v>
       </c>
+      <c r="V43" s="7" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -6943,7 +7073,7 @@
       <c r="G44" s="5" t="n">
         <v>53.8605</v>
       </c>
-      <c r="H44" s="6" t="n">
+      <c r="H44" s="5" t="n">
         <v>34.1385</v>
       </c>
       <c r="I44" s="5" t="n">
@@ -6985,6 +7115,7 @@
       <c r="U44" s="5" t="n">
         <v>-0.1632</v>
       </c>
+      <c r="V44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -7052,6 +7183,7 @@
       <c r="U45" s="5" t="n">
         <v>-0.1377</v>
       </c>
+      <c r="V45" s="7" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -7119,6 +7251,7 @@
       <c r="U46" s="5" t="n">
         <v>-0.2409</v>
       </c>
+      <c r="V46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -7186,6 +7319,7 @@
       <c r="U47" s="5" t="n">
         <v>-0.2267</v>
       </c>
+      <c r="V47" s="7" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -7253,6 +7387,7 @@
       <c r="U48" s="5" t="n">
         <v>-0.2489</v>
       </c>
+      <c r="V48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -7320,6 +7455,7 @@
       <c r="U49" s="5" t="n">
         <v>-0.3185</v>
       </c>
+      <c r="V49" s="7" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -7387,6 +7523,7 @@
       <c r="U50" s="5" t="n">
         <v>-0.3836</v>
       </c>
+      <c r="V50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -7454,6 +7591,7 @@
       <c r="U51" s="5" t="n">
         <v>-0.3384</v>
       </c>
+      <c r="V51" s="7" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -7479,7 +7617,7 @@
       <c r="G52" s="5" t="n">
         <v>52.8249</v>
       </c>
-      <c r="H52" s="6" t="n">
+      <c r="H52" s="5" t="n">
         <v>32.8876</v>
       </c>
       <c r="I52" s="5" t="n">
@@ -7521,6 +7659,7 @@
       <c r="U52" s="5" t="n">
         <v>-0.0036</v>
       </c>
+      <c r="V52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -7546,7 +7685,7 @@
       <c r="G53" s="5" t="n">
         <v>56.2122</v>
       </c>
-      <c r="H53" s="6" t="n">
+      <c r="H53" s="5" t="n">
         <v>38.4875</v>
       </c>
       <c r="I53" s="5" t="n">
@@ -7588,6 +7727,7 @@
       <c r="U53" s="5" t="n">
         <v>0.057</v>
       </c>
+      <c r="V53" s="7" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -7613,7 +7753,7 @@
       <c r="G54" s="5" t="n">
         <v>59.5995</v>
       </c>
-      <c r="H54" s="6" t="n">
+      <c r="H54" s="5" t="n">
         <v>44.4503</v>
       </c>
       <c r="I54" s="5" t="n">
@@ -7655,6 +7795,7 @@
       <c r="U54" s="5" t="n">
         <v>0.0325</v>
       </c>
+      <c r="V54" s="7" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -7722,6 +7863,7 @@
       <c r="U55" s="5" t="n">
         <v>0.0467</v>
       </c>
+      <c r="V55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -7789,6 +7931,7 @@
       <c r="U56" s="5" t="n">
         <v>0.1048</v>
       </c>
+      <c r="V56" s="7" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -7856,6 +7999,7 @@
       <c r="U57" s="5" t="n">
         <v>0.1792</v>
       </c>
+      <c r="V57" s="7" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -7923,6 +8067,7 @@
       <c r="U58" s="5" t="n">
         <v>0.1524</v>
       </c>
+      <c r="V58" s="7" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -7990,6 +8135,7 @@
       <c r="U59" s="5" t="n">
         <v>0.1704</v>
       </c>
+      <c r="V59" s="7" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -8057,6 +8203,7 @@
       <c r="U60" s="5" t="n">
         <v>0.1588</v>
       </c>
+      <c r="V60" s="7" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -8124,6 +8271,7 @@
       <c r="U61" s="5" t="n">
         <v>0.0786</v>
       </c>
+      <c r="V61" s="7" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -8149,7 +8297,7 @@
       <c r="G62" s="5" t="n">
         <v>88.39100000000001</v>
       </c>
-      <c r="H62" s="6" t="n">
+      <c r="H62" s="5" t="n">
         <v>69.8433</v>
       </c>
       <c r="I62" s="5" t="n">
@@ -8191,6 +8339,7 @@
       <c r="U62" s="5" t="n">
         <v>0.2574</v>
       </c>
+      <c r="V62" s="7" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -8216,7 +8365,7 @@
       <c r="G63" s="5" t="n">
         <v>87.6024</v>
       </c>
-      <c r="H63" s="6" t="n">
+      <c r="H63" s="5" t="n">
         <v>71.2088</v>
       </c>
       <c r="I63" s="5" t="n">
@@ -8258,6 +8407,7 @@
       <c r="U63" s="5" t="n">
         <v>0.237</v>
       </c>
+      <c r="V63" s="7" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -8283,7 +8433,7 @@
       <c r="G64" s="5" t="n">
         <v>86.8137</v>
       </c>
-      <c r="H64" s="6" t="n">
+      <c r="H64" s="5" t="n">
         <v>73.1459</v>
       </c>
       <c r="I64" s="5" t="n">
@@ -8325,6 +8475,7 @@
       <c r="U64" s="5" t="n">
         <v>0.244</v>
       </c>
+      <c r="V64" s="7" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -8392,6 +8543,7 @@
       <c r="U65" s="5" t="n">
         <v>0.2391</v>
       </c>
+      <c r="V65" s="7" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -8459,6 +8611,7 @@
       <c r="U66" s="5" t="n">
         <v>0.2399</v>
       </c>
+      <c r="V66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -8526,6 +8679,7 @@
       <c r="U67" s="5" t="n">
         <v>0.2425</v>
       </c>
+      <c r="V67" s="7" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -8593,6 +8747,7 @@
       <c r="U68" s="5" t="n">
         <v>0.3195</v>
       </c>
+      <c r="V68" s="7" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -8660,6 +8815,7 @@
       <c r="U69" s="5" t="n">
         <v>0.3255</v>
       </c>
+      <c r="V69" s="7" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -8727,6 +8883,7 @@
       <c r="U70" s="5" t="n">
         <v>0.3474</v>
       </c>
+      <c r="V70" s="7" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -8794,6 +8951,7 @@
       <c r="U71" s="5" t="n">
         <v>0.2752</v>
       </c>
+      <c r="V71" s="7" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -8819,7 +8977,7 @@
       <c r="G72" s="5" t="n">
         <v>32.981</v>
       </c>
-      <c r="H72" s="6" t="n">
+      <c r="H72" s="5" t="n">
         <v>13.3371</v>
       </c>
       <c r="I72" s="5" t="n">
@@ -8861,6 +9019,7 @@
       <c r="U72" s="5" t="n">
         <v>0.3485</v>
       </c>
+      <c r="V72" s="7" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -8886,7 +9045,7 @@
       <c r="G73" s="5" t="n">
         <v>35.209</v>
       </c>
-      <c r="H73" s="6" t="n">
+      <c r="H73" s="5" t="n">
         <v>18.1943</v>
       </c>
       <c r="I73" s="5" t="n">
@@ -8928,6 +9087,7 @@
       <c r="U73" s="5" t="n">
         <v>0.4399</v>
       </c>
+      <c r="V73" s="7" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -8953,7 +9113,7 @@
       <c r="G74" s="5" t="n">
         <v>37.4371</v>
       </c>
-      <c r="H74" s="6" t="n">
+      <c r="H74" s="5" t="n">
         <v>22.6209</v>
       </c>
       <c r="I74" s="5" t="n">
@@ -8995,6 +9155,7 @@
       <c r="U74" s="5" t="n">
         <v>0.425</v>
       </c>
+      <c r="V74" s="7" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -9062,6 +9223,7 @@
       <c r="U75" s="5" t="n">
         <v>0.5861</v>
       </c>
+      <c r="V75" s="7" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -9129,6 +9291,7 @@
       <c r="U76" s="5" t="n">
         <v>0.5753</v>
       </c>
+      <c r="V76" s="7" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -9196,6 +9359,7 @@
       <c r="U77" s="5" t="n">
         <v>0.658</v>
       </c>
+      <c r="V77" s="7" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -9263,6 +9427,7 @@
       <c r="U78" s="5" t="n">
         <v>0.5824</v>
       </c>
+      <c r="V78" s="7" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -9330,6 +9495,7 @@
       <c r="U79" s="5" t="n">
         <v>0.5338000000000001</v>
       </c>
+      <c r="V79" s="7" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -9397,6 +9563,7 @@
       <c r="U80" s="5" t="n">
         <v>0.5463</v>
       </c>
+      <c r="V80" s="7" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -9464,6 +9631,7 @@
       <c r="U81" s="5" t="n">
         <v>0.5315</v>
       </c>
+      <c r="V81" s="7" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
@@ -9489,7 +9657,7 @@
       <c r="G82" s="5" t="n">
         <v>42.1051</v>
       </c>
-      <c r="H82" s="6" t="n">
+      <c r="H82" s="5" t="n">
         <v>29.1065</v>
       </c>
       <c r="I82" s="5" t="n">
@@ -9531,6 +9699,7 @@
       <c r="U82" s="5" t="n">
         <v>-0.4487</v>
       </c>
+      <c r="V82" s="7" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -9556,7 +9725,7 @@
       <c r="G83" s="5" t="n">
         <v>46.0392</v>
       </c>
-      <c r="H83" s="6" t="n">
+      <c r="H83" s="5" t="n">
         <v>34.6304</v>
       </c>
       <c r="I83" s="5" t="n">
@@ -9598,6 +9767,7 @@
       <c r="U83" s="5" t="n">
         <v>-0.4892</v>
       </c>
+      <c r="V83" s="7" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
@@ -9623,7 +9793,7 @@
       <c r="G84" s="5" t="n">
         <v>49.9733</v>
       </c>
-      <c r="H84" s="6" t="n">
+      <c r="H84" s="5" t="n">
         <v>41.7009</v>
       </c>
       <c r="I84" s="5" t="n">
@@ -9665,6 +9835,7 @@
       <c r="U84" s="5" t="n">
         <v>-0.5085</v>
       </c>
+      <c r="V84" s="7" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -9732,6 +9903,7 @@
       <c r="U85" s="5" t="n">
         <v>-0.373</v>
       </c>
+      <c r="V85" s="7" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
@@ -9799,6 +9971,7 @@
       <c r="U86" s="5" t="n">
         <v>-0.2817</v>
       </c>
+      <c r="V86" s="7" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -9866,6 +10039,7 @@
       <c r="U87" s="5" t="n">
         <v>-0.3231</v>
       </c>
+      <c r="V87" s="7" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
@@ -9933,6 +10107,7 @@
       <c r="U88" s="5" t="n">
         <v>-0.1891</v>
       </c>
+      <c r="V88" s="7" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -10000,6 +10175,7 @@
       <c r="U89" s="5" t="n">
         <v>-0.1576</v>
       </c>
+      <c r="V89" s="7" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -10067,6 +10243,7 @@
       <c r="U90" s="5" t="n">
         <v>-0.1592</v>
       </c>
+      <c r="V90" s="7" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -10134,6 +10311,7 @@
       <c r="U91" s="5" t="n">
         <v>-0.1807</v>
       </c>
+      <c r="V91" s="7" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -10153,13 +10331,13 @@
       <c r="E92" s="5" t="n">
         <v>37.1967</v>
       </c>
-      <c r="F92" s="6" t="n">
+      <c r="F92" s="5" t="n">
         <v>18.4673</v>
       </c>
       <c r="G92" s="5" t="n">
         <v>3.7573</v>
       </c>
-      <c r="H92" s="6" t="n">
+      <c r="H92" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I92" s="5" t="n">
@@ -10201,6 +10379,7 @@
       <c r="U92" s="5" t="n">
         <v>-0.7053</v>
       </c>
+      <c r="V92" s="7" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -10220,13 +10399,13 @@
       <c r="E93" s="5" t="n">
         <v>36.9522</v>
       </c>
-      <c r="F93" s="6" t="n">
+      <c r="F93" s="5" t="n">
         <v>17.393</v>
       </c>
       <c r="G93" s="5" t="n">
         <v>8.6617</v>
       </c>
-      <c r="H93" s="6" t="n">
+      <c r="H93" s="5" t="n">
         <v>1.7866</v>
       </c>
       <c r="I93" s="5" t="n">
@@ -10268,6 +10447,7 @@
       <c r="U93" s="5" t="n">
         <v>-0.7169</v>
       </c>
+      <c r="V93" s="7" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -10287,13 +10467,13 @@
       <c r="E94" s="5" t="n">
         <v>42.1473</v>
       </c>
-      <c r="F94" s="6" t="n">
+      <c r="F94" s="5" t="n">
         <v>17.8529</v>
       </c>
       <c r="G94" s="5" t="n">
         <v>13.5662</v>
       </c>
-      <c r="H94" s="6" t="n">
+      <c r="H94" s="5" t="n">
         <v>8.2149</v>
       </c>
       <c r="I94" s="5" t="n">
@@ -10335,6 +10515,7 @@
       <c r="U94" s="5" t="n">
         <v>-0.6919</v>
       </c>
+      <c r="V94" s="7" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -10402,6 +10583,7 @@
       <c r="U95" s="5" t="n">
         <v>-0.6804</v>
       </c>
+      <c r="V95" s="7" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -10469,6 +10651,7 @@
       <c r="U96" s="5" t="n">
         <v>-0.6988</v>
       </c>
+      <c r="V96" s="7" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -10536,6 +10719,7 @@
       <c r="U97" s="5" t="n">
         <v>-0.5957</v>
       </c>
+      <c r="V97" s="7" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
@@ -10603,6 +10787,7 @@
       <c r="U98" s="5" t="n">
         <v>-0.5036</v>
       </c>
+      <c r="V98" s="7" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -10670,6 +10855,7 @@
       <c r="U99" s="5" t="n">
         <v>-0.5212</v>
       </c>
+      <c r="V99" s="7" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
@@ -10737,6 +10923,7 @@
       <c r="U100" s="5" t="n">
         <v>-0.5798</v>
       </c>
+      <c r="V100" s="7" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -10804,6 +10991,7 @@
       <c r="U101" s="5" t="n">
         <v>-0.607</v>
       </c>
+      <c r="V101" s="7" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -10829,7 +11017,7 @@
       <c r="G102" s="5" t="n">
         <v>18.0663</v>
       </c>
-      <c r="H102" s="6" t="n">
+      <c r="H102" s="5" t="n">
         <v>6.2205</v>
       </c>
       <c r="I102" s="5" t="n">
@@ -10871,6 +11059,7 @@
       <c r="U102" s="5" t="n">
         <v>-0.2379</v>
       </c>
+      <c r="V102" s="7" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -10896,7 +11085,7 @@
       <c r="G103" s="5" t="n">
         <v>17.9628</v>
       </c>
-      <c r="H103" s="6" t="n">
+      <c r="H103" s="5" t="n">
         <v>9.535500000000001</v>
       </c>
       <c r="I103" s="5" t="n">
@@ -10938,6 +11127,7 @@
       <c r="U103" s="5" t="n">
         <v>-0.3237</v>
       </c>
+      <c r="V103" s="7" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -10963,7 +11153,7 @@
       <c r="G104" s="5" t="n">
         <v>17.8592</v>
       </c>
-      <c r="H104" s="6" t="n">
+      <c r="H104" s="5" t="n">
         <v>12.0889</v>
       </c>
       <c r="I104" s="5" t="n">
@@ -11005,6 +11195,7 @@
       <c r="U104" s="5" t="n">
         <v>-0.327</v>
       </c>
+      <c r="V104" s="7" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -11072,6 +11263,7 @@
       <c r="U105" s="5" t="n">
         <v>-0.2506</v>
       </c>
+      <c r="V105" s="7" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -11139,6 +11331,7 @@
       <c r="U106" s="5" t="n">
         <v>-0.3093</v>
       </c>
+      <c r="V106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -11206,6 +11399,7 @@
       <c r="U107" s="5" t="n">
         <v>-0.328</v>
       </c>
+      <c r="V107" s="7" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -11273,6 +11467,7 @@
       <c r="U108" s="5" t="n">
         <v>-0.2777</v>
       </c>
+      <c r="V108" s="7" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -11340,6 +11535,7 @@
       <c r="U109" s="5" t="n">
         <v>-0.2948</v>
       </c>
+      <c r="V109" s="7" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -11407,6 +11603,7 @@
       <c r="U110" s="5" t="n">
         <v>-0.244</v>
       </c>
+      <c r="V110" s="7" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -11472,8 +11669,9 @@
         <v>-0.3778</v>
       </c>
       <c r="U111" s="5" t="n">
-        <v>-0.2649</v>
-      </c>
+        <v>-0.2648</v>
+      </c>
+      <c r="V111" s="7" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -11489,13 +11687,13 @@
       <c r="E112" s="5" t="n">
         <v>16.4229</v>
       </c>
-      <c r="F112" s="6" t="n">
+      <c r="F112" s="5" t="n">
         <v>16.5391</v>
       </c>
       <c r="G112" s="5" t="n">
         <v>50.438</v>
       </c>
-      <c r="H112" s="6" t="n">
+      <c r="H112" s="5" t="n">
         <v>29.9049</v>
       </c>
       <c r="I112" s="5" t="n">
@@ -11537,6 +11735,7 @@
       <c r="U112" s="5" t="n">
         <v>-0.1084</v>
       </c>
+      <c r="V112" s="7" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -11552,13 +11751,13 @@
       <c r="E113" s="5" t="n">
         <v>16.2251</v>
       </c>
-      <c r="F113" s="6" t="n">
+      <c r="F113" s="5" t="n">
         <v>17.096</v>
       </c>
       <c r="G113" s="5" t="n">
         <v>53.5673</v>
       </c>
-      <c r="H113" s="6" t="n">
+      <c r="H113" s="5" t="n">
         <v>35.8992</v>
       </c>
       <c r="I113" s="5" t="n">
@@ -11600,6 +11799,7 @@
       <c r="U113" s="5" t="n">
         <v>-0.0261</v>
       </c>
+      <c r="V113" s="7" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
@@ -11615,13 +11815,13 @@
       <c r="E114" s="5" t="n">
         <v>15.9906</v>
       </c>
-      <c r="F114" s="6" t="n">
+      <c r="F114" s="5" t="n">
         <v>16.9591</v>
       </c>
       <c r="G114" s="5" t="n">
         <v>56.6967</v>
       </c>
-      <c r="H114" s="6" t="n">
+      <c r="H114" s="5" t="n">
         <v>41.1798</v>
       </c>
       <c r="I114" s="5" t="n">
@@ -11663,6 +11863,7 @@
       <c r="U114" s="5" t="n">
         <v>0.0039</v>
       </c>
+      <c r="V114" s="7" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -11678,7 +11879,7 @@
       <c r="E115" s="5" t="n">
         <v>18.8501</v>
       </c>
-      <c r="F115" s="6" t="n">
+      <c r="F115" s="5" t="n">
         <v>16.885</v>
       </c>
       <c r="G115" s="5" t="n">
@@ -11726,6 +11927,7 @@
       <c r="U115" s="5" t="n">
         <v>0.0912</v>
       </c>
+      <c r="V115" s="7" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -11741,7 +11943,7 @@
       <c r="E116" s="5" t="n">
         <v>20.882</v>
       </c>
-      <c r="F116" s="6" t="n">
+      <c r="F116" s="5" t="n">
         <v>17.634</v>
       </c>
       <c r="G116" s="5" t="n">
@@ -11789,6 +11991,7 @@
       <c r="U116" s="5" t="n">
         <v>0.1241</v>
       </c>
+      <c r="V116" s="7" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -11804,7 +12007,7 @@
       <c r="E117" s="5" t="n">
         <v>21.474</v>
       </c>
-      <c r="F117" s="6" t="n">
+      <c r="F117" s="5" t="n">
         <v>17.9061</v>
       </c>
       <c r="G117" s="5" t="n">
@@ -11852,6 +12055,7 @@
       <c r="U117" s="5" t="n">
         <v>0.117</v>
       </c>
+      <c r="V117" s="7" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -11867,7 +12071,7 @@
       <c r="E118" s="5" t="n">
         <v>21.975</v>
       </c>
-      <c r="F118" s="6" t="n">
+      <c r="F118" s="5" t="n">
         <v>18.3306</v>
       </c>
       <c r="G118" s="5" t="n">
@@ -11915,6 +12119,7 @@
       <c r="U118" s="5" t="n">
         <v>0.13</v>
       </c>
+      <c r="V118" s="7" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -11930,13 +12135,13 @@
       <c r="E119" s="5" t="n">
         <v>21.8619</v>
       </c>
-      <c r="F119" s="6" t="n">
+      <c r="F119" s="5" t="n">
         <v>18.5032</v>
       </c>
-      <c r="G119" s="6" t="n">
+      <c r="G119" s="5" t="n">
         <v>73.32429999999999</v>
       </c>
-      <c r="H119" s="6" t="n">
+      <c r="H119" s="5" t="n">
         <v>63.0555</v>
       </c>
       <c r="I119" s="5" t="n">
@@ -11978,6 +12183,7 @@
       <c r="U119" s="5" t="n">
         <v>0.1788</v>
       </c>
+      <c r="V119" s="7" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="inlineStr">
@@ -11993,13 +12199,13 @@
       <c r="E120" s="5" t="n">
         <v>20.5907</v>
       </c>
-      <c r="F120" s="6" t="n">
+      <c r="F120" s="5" t="n">
         <v>18.2432</v>
       </c>
-      <c r="G120" s="6" t="n">
+      <c r="G120" s="5" t="n">
         <v>77.6698</v>
       </c>
-      <c r="H120" s="6" t="n">
+      <c r="H120" s="5" t="n">
         <v>67.60250000000001</v>
       </c>
       <c r="I120" s="5" t="n">
@@ -12041,6 +12247,7 @@
       <c r="U120" s="5" t="n">
         <v>0.1865</v>
       </c>
+      <c r="V120" s="7" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="inlineStr">
@@ -12056,13 +12263,13 @@
       <c r="E121" s="5" t="n">
         <v>21.5238</v>
       </c>
-      <c r="F121" s="6" t="n">
+      <c r="F121" s="5" t="n">
         <v>17.3562</v>
       </c>
-      <c r="G121" s="6" t="n">
+      <c r="G121" s="5" t="n">
         <v>84.8143</v>
       </c>
-      <c r="H121" s="6" t="n">
+      <c r="H121" s="5" t="n">
         <v>72.4139</v>
       </c>
       <c r="I121" s="5" t="n">
@@ -12104,6 +12311,7 @@
       <c r="U121" s="5" t="n">
         <v>0.1799</v>
       </c>
+      <c r="V121" s="7" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="inlineStr">
@@ -12129,7 +12337,7 @@
       <c r="G122" s="5" t="n">
         <v>73.69889999999999</v>
       </c>
-      <c r="H122" s="6" t="n">
+      <c r="H122" s="5" t="n">
         <v>48.8509</v>
       </c>
       <c r="I122" s="5" t="n">
@@ -12171,6 +12379,7 @@
       <c r="U122" s="5" t="n">
         <v>-0.2372</v>
       </c>
+      <c r="V122" s="7" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="inlineStr">
@@ -12196,7 +12405,7 @@
       <c r="G123" s="5" t="n">
         <v>73.0654</v>
       </c>
-      <c r="H123" s="6" t="n">
+      <c r="H123" s="5" t="n">
         <v>50.1393</v>
       </c>
       <c r="I123" s="5" t="n">
@@ -12238,6 +12447,7 @@
       <c r="U123" s="5" t="n">
         <v>0.0098</v>
       </c>
+      <c r="V123" s="7" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -12263,7 +12473,7 @@
       <c r="G124" s="5" t="n">
         <v>72.432</v>
       </c>
-      <c r="H124" s="6" t="n">
+      <c r="H124" s="5" t="n">
         <v>52.3241</v>
       </c>
       <c r="I124" s="5" t="n">
@@ -12305,6 +12515,7 @@
       <c r="U124" s="5" t="n">
         <v>-0.0278</v>
       </c>
+      <c r="V124" s="7" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -12370,8 +12581,9 @@
         <v>-0.1921</v>
       </c>
       <c r="U125" s="5" t="n">
-        <v>0.0441</v>
-      </c>
+        <v>0.044</v>
+      </c>
+      <c r="V125" s="7" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -12439,6 +12651,7 @@
       <c r="U126" s="5" t="n">
         <v>-0.0038</v>
       </c>
+      <c r="V126" s="7" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="inlineStr">
@@ -12504,8 +12717,9 @@
         <v>-0.3194</v>
       </c>
       <c r="U127" s="5" t="n">
-        <v>-0.0227</v>
-      </c>
+        <v>-0.0226</v>
+      </c>
+      <c r="V127" s="7" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -12573,6 +12787,7 @@
       <c r="U128" s="5" t="n">
         <v>0.0141</v>
       </c>
+      <c r="V128" s="7" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -12640,6 +12855,7 @@
       <c r="U129" s="5" t="n">
         <v>0.08599999999999999</v>
       </c>
+      <c r="V129" s="7" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="inlineStr">
@@ -12707,6 +12923,7 @@
       <c r="U130" s="5" t="n">
         <v>-0.0467</v>
       </c>
+      <c r="V130" s="7" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="inlineStr">
@@ -12774,6 +12991,7 @@
       <c r="U131" s="5" t="n">
         <v>0.06519999999999999</v>
       </c>
+      <c r="V131" s="7" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="inlineStr">
@@ -12799,7 +13017,7 @@
       <c r="G132" s="5" t="n">
         <v>44.5916</v>
       </c>
-      <c r="H132" s="6" t="n">
+      <c r="H132" s="5" t="n">
         <v>22.1137</v>
       </c>
       <c r="I132" s="5" t="n">
@@ -12841,6 +13059,7 @@
       <c r="U132" s="5" t="n">
         <v>0.2635</v>
       </c>
+      <c r="V132" s="7" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="inlineStr">
@@ -12866,7 +13085,7 @@
       <c r="G133" s="5" t="n">
         <v>50.0068</v>
       </c>
-      <c r="H133" s="6" t="n">
+      <c r="H133" s="5" t="n">
         <v>30.3369</v>
       </c>
       <c r="I133" s="5" t="n">
@@ -12908,6 +13127,7 @@
       <c r="U133" s="5" t="n">
         <v>0.2273</v>
       </c>
+      <c r="V133" s="7" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="inlineStr">
@@ -12933,7 +13153,7 @@
       <c r="G134" s="5" t="n">
         <v>55.422</v>
       </c>
-      <c r="H134" s="6" t="n">
+      <c r="H134" s="5" t="n">
         <v>38.0707</v>
       </c>
       <c r="I134" s="5" t="n">
@@ -12975,6 +13195,7 @@
       <c r="U134" s="5" t="n">
         <v>0.2973</v>
       </c>
+      <c r="V134" s="7" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="inlineStr">
@@ -13042,6 +13263,7 @@
       <c r="U135" s="5" t="n">
         <v>0.3765</v>
       </c>
+      <c r="V135" s="7" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="inlineStr">
@@ -13109,6 +13331,7 @@
       <c r="U136" s="5" t="n">
         <v>0.4192</v>
       </c>
+      <c r="V136" s="7" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="inlineStr">
@@ -13176,6 +13399,7 @@
       <c r="U137" s="5" t="n">
         <v>0.4088</v>
       </c>
+      <c r="V137" s="7" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="inlineStr">
@@ -13243,6 +13467,7 @@
       <c r="U138" s="5" t="n">
         <v>0.4075</v>
       </c>
+      <c r="V138" s="7" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -13310,6 +13535,7 @@
       <c r="U139" s="5" t="n">
         <v>0.3461</v>
       </c>
+      <c r="V139" s="7" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="inlineStr">
@@ -13377,6 +13603,7 @@
       <c r="U140" s="5" t="n">
         <v>0.362</v>
       </c>
+      <c r="V140" s="7" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -13444,6 +13671,7 @@
       <c r="U141" s="5" t="n">
         <v>0.381</v>
       </c>
+      <c r="V141" s="7" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="inlineStr">
@@ -13469,7 +13697,7 @@
       <c r="G142" s="5" t="n">
         <v>48.1785</v>
       </c>
-      <c r="H142" s="6" t="n">
+      <c r="H142" s="5" t="n">
         <v>35.5388</v>
       </c>
       <c r="I142" s="5" t="n">
@@ -13511,6 +13739,7 @@
       <c r="U142" s="5" t="n">
         <v>-0.5332</v>
       </c>
+      <c r="V142" s="7" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -13536,7 +13765,7 @@
       <c r="G143" s="5" t="n">
         <v>54.58</v>
       </c>
-      <c r="H143" s="6" t="n">
+      <c r="H143" s="5" t="n">
         <v>44.7348</v>
       </c>
       <c r="I143" s="5" t="n">
@@ -13578,6 +13807,7 @@
       <c r="U143" s="5" t="n">
         <v>-0.6985</v>
       </c>
+      <c r="V143" s="7" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="inlineStr">
@@ -13603,7 +13833,7 @@
       <c r="G144" s="5" t="n">
         <v>60.9816</v>
       </c>
-      <c r="H144" s="6" t="n">
+      <c r="H144" s="5" t="n">
         <v>52.1422</v>
       </c>
       <c r="I144" s="5" t="n">
@@ -13645,6 +13875,7 @@
       <c r="U144" s="5" t="n">
         <v>-0.6604</v>
       </c>
+      <c r="V144" s="7" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="inlineStr">
@@ -13712,6 +13943,7 @@
       <c r="U145" s="5" t="n">
         <v>-0.6514</v>
       </c>
+      <c r="V145" s="7" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -13779,6 +14011,7 @@
       <c r="U146" s="5" t="n">
         <v>-0.7122000000000001</v>
       </c>
+      <c r="V146" s="7" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -13846,6 +14079,7 @@
       <c r="U147" s="5" t="n">
         <v>-0.6457000000000001</v>
       </c>
+      <c r="V147" s="7" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -13913,6 +14147,7 @@
       <c r="U148" s="5" t="n">
         <v>-0.6169</v>
       </c>
+      <c r="V148" s="7" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -13980,6 +14215,7 @@
       <c r="U149" s="5" t="n">
         <v>-0.5951</v>
       </c>
+      <c r="V149" s="7" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -14047,6 +14283,7 @@
       <c r="U150" s="5" t="n">
         <v>-0.6105</v>
       </c>
+      <c r="V150" s="7" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
@@ -14114,6 +14351,7 @@
       <c r="U151" s="5" t="n">
         <v>-0.6352</v>
       </c>
+      <c r="V151" s="7" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="inlineStr">
@@ -14135,7 +14373,7 @@
       <c r="G152" s="5" t="n">
         <v>62.2162</v>
       </c>
-      <c r="H152" s="6" t="n">
+      <c r="H152" s="5" t="n">
         <v>40.9977</v>
       </c>
       <c r="I152" s="5" t="n">
@@ -14177,6 +14415,7 @@
       <c r="U152" s="5" t="n">
         <v>-0.2549</v>
       </c>
+      <c r="V152" s="7" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -14198,7 +14437,7 @@
       <c r="G153" s="5" t="n">
         <v>69.17489999999999</v>
       </c>
-      <c r="H153" s="6" t="n">
+      <c r="H153" s="5" t="n">
         <v>50.1173</v>
       </c>
       <c r="I153" s="5" t="n">
@@ -14240,6 +14479,7 @@
       <c r="U153" s="5" t="n">
         <v>-0.2451</v>
       </c>
+      <c r="V153" s="7" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -14261,7 +14501,7 @@
       <c r="G154" s="5" t="n">
         <v>76.1336</v>
       </c>
-      <c r="H154" s="6" t="n">
+      <c r="H154" s="5" t="n">
         <v>59.868</v>
       </c>
       <c r="I154" s="5" t="n">
@@ -14303,6 +14543,7 @@
       <c r="U154" s="5" t="n">
         <v>-0.226</v>
       </c>
+      <c r="V154" s="7" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -14366,6 +14607,7 @@
       <c r="U155" s="5" t="n">
         <v>-0.0344</v>
       </c>
+      <c r="V155" s="7" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -14429,6 +14671,7 @@
       <c r="U156" s="5" t="n">
         <v>0.0193</v>
       </c>
+      <c r="V156" s="7" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -14492,6 +14735,7 @@
       <c r="U157" s="5" t="n">
         <v>-0.0391</v>
       </c>
+      <c r="V157" s="7" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -14555,6 +14799,7 @@
       <c r="U158" s="5" t="n">
         <v>-0.0412</v>
       </c>
+      <c r="V158" s="7" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -14618,6 +14863,7 @@
       <c r="U159" s="5" t="n">
         <v>-0.0051</v>
       </c>
+      <c r="V159" s="7" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -14681,6 +14927,7 @@
       <c r="U160" s="5" t="n">
         <v>-0.0005</v>
       </c>
+      <c r="V160" s="7" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -14744,6 +14991,7 @@
       <c r="U161" s="5" t="n">
         <v>-0.0348</v>
       </c>
+      <c r="V161" s="7" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -14769,7 +15017,7 @@
       <c r="G162" s="5" t="n">
         <v>2.5349</v>
       </c>
-      <c r="H162" s="6" t="n">
+      <c r="H162" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I162" s="5" t="n">
@@ -14811,6 +15059,7 @@
       <c r="U162" s="5" t="n">
         <v>-1.1105</v>
       </c>
+      <c r="V162" s="7" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -14836,7 +15085,7 @@
       <c r="G163" s="5" t="n">
         <v>5.5097</v>
       </c>
-      <c r="H163" s="6" t="n">
+      <c r="H163" s="5" t="n">
         <v>0.9954</v>
       </c>
       <c r="I163" s="5" t="n">
@@ -14878,6 +15127,7 @@
       <c r="U163" s="5" t="n">
         <v>-1.0899</v>
       </c>
+      <c r="V163" s="7" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -14903,7 +15153,7 @@
       <c r="G164" s="5" t="n">
         <v>8.484400000000001</v>
       </c>
-      <c r="H164" s="6" t="n">
+      <c r="H164" s="5" t="n">
         <v>6.4301</v>
       </c>
       <c r="I164" s="5" t="n">
@@ -14945,6 +15195,7 @@
       <c r="U164" s="5" t="n">
         <v>-1.1126</v>
       </c>
+      <c r="V164" s="7" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="inlineStr">
@@ -15012,6 +15263,7 @@
       <c r="U165" s="5" t="n">
         <v>-1.041</v>
       </c>
+      <c r="V165" s="7" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="inlineStr">
@@ -15079,6 +15331,7 @@
       <c r="U166" s="5" t="n">
         <v>-1.0065</v>
       </c>
+      <c r="V166" s="7" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="inlineStr">
@@ -15146,6 +15399,7 @@
       <c r="U167" s="5" t="n">
         <v>-1.0278</v>
       </c>
+      <c r="V167" s="7" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="inlineStr">
@@ -15189,7 +15443,7 @@
       <c r="M168" s="5" t="n">
         <v>7.035</v>
       </c>
-      <c r="N168" s="6" t="n">
+      <c r="N168" s="5" t="n">
         <v>6.8918</v>
       </c>
       <c r="O168" s="5" t="n">
@@ -15211,8 +15465,9 @@
         <v>-1.1642</v>
       </c>
       <c r="U168" s="5" t="n">
-        <v>-0.9774</v>
-      </c>
+        <v>-0.9775</v>
+      </c>
+      <c r="V168" s="7" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -15256,7 +15511,7 @@
       <c r="M169" s="5" t="n">
         <v>7.028</v>
       </c>
-      <c r="N169" s="6" t="n">
+      <c r="N169" s="5" t="n">
         <v>7.1192</v>
       </c>
       <c r="O169" s="5" t="n">
@@ -15280,6 +15535,7 @@
       <c r="U169" s="5" t="n">
         <v>-0.9348</v>
       </c>
+      <c r="V169" s="7" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="inlineStr">
@@ -15323,7 +15579,7 @@
       <c r="M170" s="5" t="n">
         <v>7.026</v>
       </c>
-      <c r="N170" s="6" t="n">
+      <c r="N170" s="5" t="n">
         <v>6.5756</v>
       </c>
       <c r="O170" s="5" t="n">
@@ -15347,6 +15603,7 @@
       <c r="U170" s="5" t="n">
         <v>-1.0236</v>
       </c>
+      <c r="V170" s="7" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="inlineStr">
@@ -15390,7 +15647,7 @@
       <c r="M171" s="5" t="n">
         <v>7.576</v>
       </c>
-      <c r="N171" s="6" t="n">
+      <c r="N171" s="5" t="n">
         <v>8.811299999999999</v>
       </c>
       <c r="O171" s="5" t="n">
@@ -15414,6 +15671,7 @@
       <c r="U171" s="5" t="n">
         <v>-1.0238</v>
       </c>
+      <c r="V171" s="7" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
@@ -15429,16 +15687,16 @@
       <c r="E172" s="5" t="n">
         <v>36.7918</v>
       </c>
-      <c r="F172" s="6" t="n">
+      <c r="F172" s="5" t="n">
         <v>13.3357</v>
       </c>
       <c r="G172" s="5" t="n">
         <v>0.4049</v>
       </c>
-      <c r="H172" s="6" t="n">
+      <c r="H172" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="I172" s="6" t="n">
+      <c r="I172" s="5" t="n">
         <v>32.7746</v>
       </c>
       <c r="J172" s="5" t="n">
@@ -15453,10 +15711,10 @@
       <c r="M172" s="5" t="n">
         <v>4.003</v>
       </c>
-      <c r="N172" s="6" t="n">
+      <c r="N172" s="5" t="n">
         <v>15.1678</v>
       </c>
-      <c r="O172" s="6" t="n">
+      <c r="O172" s="5" t="n">
         <v>16.059</v>
       </c>
       <c r="P172" s="5" t="n">
@@ -15477,6 +15735,7 @@
       <c r="U172" s="5" t="n">
         <v>-1.626</v>
       </c>
+      <c r="V172" s="7" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="inlineStr">
@@ -15492,16 +15751,16 @@
       <c r="E173" s="5" t="n">
         <v>36.2132</v>
       </c>
-      <c r="F173" s="6" t="n">
+      <c r="F173" s="5" t="n">
         <v>12.4057</v>
       </c>
       <c r="G173" s="5" t="n">
         <v>7.1002</v>
       </c>
-      <c r="H173" s="6" t="n">
+      <c r="H173" s="5" t="n">
         <v>0.0716</v>
       </c>
-      <c r="I173" s="6" t="n">
+      <c r="I173" s="5" t="n">
         <v>46.6004</v>
       </c>
       <c r="J173" s="5" t="n">
@@ -15516,10 +15775,10 @@
       <c r="M173" s="5" t="n">
         <v>3.994</v>
       </c>
-      <c r="N173" s="6" t="n">
+      <c r="N173" s="5" t="n">
         <v>13.397</v>
       </c>
-      <c r="O173" s="6" t="n">
+      <c r="O173" s="5" t="n">
         <v>11.2022</v>
       </c>
       <c r="P173" s="5" t="n">
@@ -15540,6 +15799,7 @@
       <c r="U173" s="5" t="n">
         <v>-1.6012</v>
       </c>
+      <c r="V173" s="7" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
@@ -15555,16 +15815,16 @@
       <c r="E174" s="5" t="n">
         <v>35.6764</v>
       </c>
-      <c r="F174" s="6" t="n">
+      <c r="F174" s="5" t="n">
         <v>12.0033</v>
       </c>
       <c r="G174" s="5" t="n">
         <v>13.7954</v>
       </c>
-      <c r="H174" s="6" t="n">
+      <c r="H174" s="5" t="n">
         <v>8.244300000000001</v>
       </c>
-      <c r="I174" s="6" t="n">
+      <c r="I174" s="5" t="n">
         <v>50.934</v>
       </c>
       <c r="J174" s="5" t="n">
@@ -15579,10 +15839,10 @@
       <c r="M174" s="5" t="n">
         <v>3.993</v>
       </c>
-      <c r="N174" s="6" t="n">
+      <c r="N174" s="5" t="n">
         <v>12.4992</v>
       </c>
-      <c r="O174" s="6" t="n">
+      <c r="O174" s="5" t="n">
         <v>9.594200000000001</v>
       </c>
       <c r="P174" s="5" t="n">
@@ -15603,6 +15863,7 @@
       <c r="U174" s="5" t="n">
         <v>-1.6093</v>
       </c>
+      <c r="V174" s="7" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
@@ -15618,16 +15879,16 @@
       <c r="E175" s="5" t="n">
         <v>35.1884</v>
       </c>
-      <c r="F175" s="6" t="n">
+      <c r="F175" s="5" t="n">
         <v>11.7729</v>
       </c>
       <c r="G175" s="5" t="n">
-        <v>20.4907</v>
-      </c>
-      <c r="H175" s="6" t="n">
+        <v>20.4906</v>
+      </c>
+      <c r="H175" s="5" t="n">
         <v>15.7366</v>
       </c>
-      <c r="I175" s="6" t="n">
+      <c r="I175" s="5" t="n">
         <v>58.6619</v>
       </c>
       <c r="J175" s="5" t="n">
@@ -15642,10 +15903,10 @@
       <c r="M175" s="5" t="n">
         <v>4.005</v>
       </c>
-      <c r="N175" s="6" t="n">
+      <c r="N175" s="5" t="n">
         <v>10.7845</v>
       </c>
-      <c r="O175" s="6" t="n">
+      <c r="O175" s="5" t="n">
         <v>8.1601</v>
       </c>
       <c r="P175" s="5" t="n">
@@ -15666,6 +15927,7 @@
       <c r="U175" s="5" t="n">
         <v>-1.5953</v>
       </c>
+      <c r="V175" s="7" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
@@ -15681,16 +15943,16 @@
       <c r="E176" s="5" t="n">
         <v>34.7667</v>
       </c>
-      <c r="F176" s="6" t="n">
+      <c r="F176" s="5" t="n">
         <v>10.3611</v>
       </c>
       <c r="G176" s="5" t="n">
         <v>27.1859</v>
       </c>
-      <c r="H176" s="6" t="n">
+      <c r="H176" s="5" t="n">
         <v>22.6067</v>
       </c>
-      <c r="I176" s="6" t="n">
+      <c r="I176" s="5" t="n">
         <v>62.9422</v>
       </c>
       <c r="J176" s="5" t="n">
@@ -15705,10 +15967,10 @@
       <c r="M176" s="5" t="n">
         <v>4.016</v>
       </c>
-      <c r="N176" s="6" t="n">
+      <c r="N176" s="5" t="n">
         <v>8.9725</v>
       </c>
-      <c r="O176" s="6" t="n">
+      <c r="O176" s="5" t="n">
         <v>6.828</v>
       </c>
       <c r="P176" s="5" t="n">
@@ -15729,6 +15991,7 @@
       <c r="U176" s="5" t="n">
         <v>-1.5898</v>
       </c>
+      <c r="V176" s="7" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -15744,16 +16007,16 @@
       <c r="E177" s="5" t="n">
         <v>34.4187</v>
       </c>
-      <c r="F177" s="6" t="n">
+      <c r="F177" s="5" t="n">
         <v>9.5541</v>
       </c>
       <c r="G177" s="5" t="n">
         <v>33.8811</v>
       </c>
-      <c r="H177" s="6" t="n">
+      <c r="H177" s="5" t="n">
         <v>29.4543</v>
       </c>
-      <c r="I177" s="6" t="n">
+      <c r="I177" s="5" t="n">
         <v>67.3305</v>
       </c>
       <c r="J177" s="5" t="n">
@@ -15768,10 +16031,10 @@
       <c r="M177" s="5" t="n">
         <v>4.026</v>
       </c>
-      <c r="N177" s="6" t="n">
+      <c r="N177" s="5" t="n">
         <v>7.6891</v>
       </c>
-      <c r="O177" s="6" t="n">
+      <c r="O177" s="5" t="n">
         <v>5.4267</v>
       </c>
       <c r="P177" s="5" t="n">
@@ -15792,6 +16055,7 @@
       <c r="U177" s="5" t="n">
         <v>-1.6315</v>
       </c>
+      <c r="V177" s="7" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
@@ -15807,7 +16071,7 @@
       <c r="E178" s="5" t="n">
         <v>34.1184</v>
       </c>
-      <c r="F178" s="6" t="n">
+      <c r="F178" s="5" t="n">
         <v>8.6493</v>
       </c>
       <c r="G178" s="5" t="n">
@@ -15816,7 +16080,7 @@
       <c r="H178" s="5" t="n">
         <v>34.2975</v>
       </c>
-      <c r="I178" s="6" t="n">
+      <c r="I178" s="5" t="n">
         <v>66.99209999999999</v>
       </c>
       <c r="J178" s="5" t="n">
@@ -15831,10 +16095,10 @@
       <c r="M178" s="5" t="n">
         <v>4.035</v>
       </c>
-      <c r="N178" s="6" t="n">
+      <c r="N178" s="5" t="n">
         <v>8.504300000000001</v>
       </c>
-      <c r="O178" s="6" t="n">
+      <c r="O178" s="5" t="n">
         <v>3.1227</v>
       </c>
       <c r="P178" s="5" t="n">
@@ -15855,6 +16119,7 @@
       <c r="U178" s="5" t="n">
         <v>-1.6343</v>
       </c>
+      <c r="V178" s="7" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -15870,16 +16135,16 @@
       <c r="E179" s="5" t="n">
         <v>33.8603</v>
       </c>
-      <c r="F179" s="6" t="n">
+      <c r="F179" s="5" t="n">
         <v>8.2174</v>
       </c>
-      <c r="G179" s="6" t="n">
+      <c r="G179" s="5" t="n">
         <v>36.409</v>
       </c>
-      <c r="H179" s="6" t="n">
+      <c r="H179" s="5" t="n">
         <v>34.0764</v>
       </c>
-      <c r="I179" s="6" t="n">
+      <c r="I179" s="5" t="n">
         <v>61.4315</v>
       </c>
       <c r="J179" s="5" t="n">
@@ -15894,10 +16159,10 @@
       <c r="M179" s="5" t="n">
         <v>4.036</v>
       </c>
-      <c r="N179" s="6" t="n">
+      <c r="N179" s="5" t="n">
         <v>9.9893</v>
       </c>
-      <c r="O179" s="6" t="n">
+      <c r="O179" s="5" t="n">
         <v>5.1014</v>
       </c>
       <c r="P179" s="5" t="n">
@@ -15918,6 +16183,7 @@
       <c r="U179" s="5" t="n">
         <v>-1.621</v>
       </c>
+      <c r="V179" s="7" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="inlineStr">
@@ -15933,16 +16199,16 @@
       <c r="E180" s="5" t="n">
         <v>33.6193</v>
       </c>
-      <c r="F180" s="6" t="n">
+      <c r="F180" s="5" t="n">
         <v>7.6099</v>
       </c>
-      <c r="G180" s="6" t="n">
+      <c r="G180" s="5" t="n">
         <v>39.4864</v>
       </c>
-      <c r="H180" s="6" t="n">
+      <c r="H180" s="5" t="n">
         <v>37.0783</v>
       </c>
-      <c r="I180" s="6" t="n">
+      <c r="I180" s="5" t="n">
         <v>64.5491</v>
       </c>
       <c r="J180" s="5" t="n">
@@ -15957,10 +16223,10 @@
       <c r="M180" s="5" t="n">
         <v>4.035</v>
       </c>
-      <c r="N180" s="6" t="n">
+      <c r="N180" s="5" t="n">
         <v>9.6957</v>
       </c>
-      <c r="O180" s="6" t="n">
+      <c r="O180" s="5" t="n">
         <v>4.7529</v>
       </c>
       <c r="P180" s="5" t="n">
@@ -15981,6 +16247,7 @@
       <c r="U180" s="5" t="n">
         <v>-1.6521</v>
       </c>
+      <c r="V180" s="7" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="inlineStr">
@@ -15996,16 +16263,16 @@
       <c r="E181" s="5" t="n">
         <v>33.0787</v>
       </c>
-      <c r="F181" s="6" t="n">
+      <c r="F181" s="5" t="n">
         <v>7.1927</v>
       </c>
-      <c r="G181" s="6" t="n">
+      <c r="G181" s="5" t="n">
         <v>44.2236</v>
       </c>
-      <c r="H181" s="6" t="n">
+      <c r="H181" s="5" t="n">
         <v>40.7546</v>
       </c>
-      <c r="I181" s="6" t="n">
+      <c r="I181" s="5" t="n">
         <v>66.2795</v>
       </c>
       <c r="J181" s="5" t="n">
@@ -16020,10 +16287,10 @@
       <c r="M181" s="5" t="n">
         <v>4.489</v>
       </c>
-      <c r="N181" s="6" t="n">
+      <c r="N181" s="5" t="n">
         <v>9.2835</v>
       </c>
-      <c r="O181" s="6" t="n">
+      <c r="O181" s="5" t="n">
         <v>4.17</v>
       </c>
       <c r="P181" s="5" t="n">
@@ -16044,6 +16311,7 @@
       <c r="U181" s="5" t="n">
         <v>-1.6206</v>
       </c>
+      <c r="V181" s="7" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="inlineStr">
@@ -16069,7 +16337,7 @@
       <c r="G182" s="5" t="n">
         <v>41.2686</v>
       </c>
-      <c r="H182" s="6" t="n">
+      <c r="H182" s="5" t="n">
         <v>30.4485</v>
       </c>
       <c r="I182" s="5" t="n">
@@ -16111,6 +16379,7 @@
       <c r="U182" s="5" t="n">
         <v>-0.7802</v>
       </c>
+      <c r="V182" s="7" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="inlineStr">
@@ -16136,7 +16405,7 @@
       <c r="G183" s="5" t="n">
         <v>45.084</v>
       </c>
-      <c r="H183" s="6" t="n">
+      <c r="H183" s="5" t="n">
         <v>36.1729</v>
       </c>
       <c r="I183" s="5" t="n">
@@ -16178,6 +16447,7 @@
       <c r="U183" s="5" t="n">
         <v>-0.6827</v>
       </c>
+      <c r="V183" s="7" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
@@ -16203,7 +16473,7 @@
       <c r="G184" s="5" t="n">
         <v>48.8994</v>
       </c>
-      <c r="H184" s="6" t="n">
+      <c r="H184" s="5" t="n">
         <v>41.7189</v>
       </c>
       <c r="I184" s="5" t="n">
@@ -16245,6 +16515,7 @@
       <c r="U184" s="5" t="n">
         <v>-0.6935</v>
       </c>
+      <c r="V184" s="7" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="inlineStr">
@@ -16312,6 +16583,7 @@
       <c r="U185" s="5" t="n">
         <v>-0.6742</v>
       </c>
+      <c r="V185" s="7" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="inlineStr">
@@ -16379,6 +16651,7 @@
       <c r="U186" s="5" t="n">
         <v>-0.6584</v>
       </c>
+      <c r="V186" s="7" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -16446,6 +16719,7 @@
       <c r="U187" s="5" t="n">
         <v>-0.584</v>
       </c>
+      <c r="V187" s="7" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="inlineStr">
@@ -16513,6 +16787,7 @@
       <c r="U188" s="5" t="n">
         <v>-0.4722</v>
       </c>
+      <c r="V188" s="7" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="inlineStr">
@@ -16580,6 +16855,7 @@
       <c r="U189" s="5" t="n">
         <v>-0.4335</v>
       </c>
+      <c r="V189" s="7" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="inlineStr">
@@ -16647,6 +16923,7 @@
       <c r="U190" s="5" t="n">
         <v>-0.4378</v>
       </c>
+      <c r="V190" s="7" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -16714,6 +16991,7 @@
       <c r="U191" s="5" t="n">
         <v>-0.4583</v>
       </c>
+      <c r="V191" s="7" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="inlineStr">
@@ -16735,10 +17013,10 @@
       <c r="G192" s="5" t="n">
         <v>22.5039</v>
       </c>
-      <c r="H192" s="6" t="n">
+      <c r="H192" s="5" t="n">
         <v>11.3162</v>
       </c>
-      <c r="I192" s="6" t="n">
+      <c r="I192" s="5" t="n">
         <v>18.8115</v>
       </c>
       <c r="J192" s="5" t="n">
@@ -16776,6 +17054,9 @@
       </c>
       <c r="U192" s="5" t="n">
         <v>-1.472</v>
+      </c>
+      <c r="V192" s="8" t="n">
+        <v>7.57</v>
       </c>
     </row>
     <row r="193">
@@ -16798,10 +17079,10 @@
       <c r="G193" s="5" t="n">
         <v>28.5726</v>
       </c>
-      <c r="H193" s="6" t="n">
+      <c r="H193" s="5" t="n">
         <v>19.7963</v>
       </c>
-      <c r="I193" s="6" t="n">
+      <c r="I193" s="5" t="n">
         <v>17.9086</v>
       </c>
       <c r="J193" s="5" t="n">
@@ -16839,6 +17120,9 @@
       </c>
       <c r="U193" s="5" t="n">
         <v>-1.3248</v>
+      </c>
+      <c r="V193" s="8" t="n">
+        <v>7.33</v>
       </c>
     </row>
     <row r="194">
@@ -16861,10 +17145,10 @@
       <c r="G194" s="5" t="n">
         <v>34.6413</v>
       </c>
-      <c r="H194" s="6" t="n">
+      <c r="H194" s="5" t="n">
         <v>27.5603</v>
       </c>
-      <c r="I194" s="6" t="n">
+      <c r="I194" s="5" t="n">
         <v>21.0419</v>
       </c>
       <c r="J194" s="5" t="n">
@@ -16902,6 +17186,9 @@
       </c>
       <c r="U194" s="5" t="n">
         <v>-1.2945</v>
+      </c>
+      <c r="V194" s="8" t="n">
+        <v>8.02</v>
       </c>
     </row>
     <row r="195">
@@ -16966,6 +17253,9 @@
       <c r="U195" s="5" t="n">
         <v>-1.2757</v>
       </c>
+      <c r="V195" s="8" t="n">
+        <v>8.119999999999999</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="4" t="inlineStr">
@@ -17029,6 +17319,9 @@
       <c r="U196" s="5" t="n">
         <v>-1.2503</v>
       </c>
+      <c r="V196" s="8" t="n">
+        <v>7.63</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -17092,6 +17385,9 @@
       <c r="U197" s="5" t="n">
         <v>-1.2217</v>
       </c>
+      <c r="V197" s="8" t="n">
+        <v>7.66</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -17155,6 +17451,9 @@
       <c r="U198" s="5" t="n">
         <v>-1.1445</v>
       </c>
+      <c r="V198" s="8" t="n">
+        <v>6.99</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="4" t="inlineStr">
@@ -17218,6 +17517,9 @@
       <c r="U199" s="5" t="n">
         <v>-1.0216</v>
       </c>
+      <c r="V199" s="8" t="n">
+        <v>6.88</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="4" t="inlineStr">
@@ -17281,6 +17583,9 @@
       <c r="U200" s="5" t="n">
         <v>-0.9327</v>
       </c>
+      <c r="V200" s="8" t="n">
+        <v>7.43</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
@@ -17342,7 +17647,10 @@
         <v>-0.9126</v>
       </c>
       <c r="U201" s="5" t="n">
-        <v>-0.9675</v>
+        <v>-0.9676</v>
+      </c>
+      <c r="V201" s="8" t="n">
+        <v>6.49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>